<commit_message>
Polish sending: HTML email body, Iqama password, compact visual UI
- .eml drafts now carry a multipart/alternative body (plain + HTML with
  real paragraphs) so Outlook keeps the line breaks; shorter default
  message: greeting, one line, password, company
- default PDF password is the Iqama / National ID number with a one-line
  hint; other rules remain available
- UI: shorter copy throughout, icon-based three-step flows per channel
  instead of paragraphs, stepper with ticks and progress line, panel
  fade-in, hover lift, striped progress bar, reduced-motion respected

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016bCq81BBBapftKyzt9FyKX
</commit_message>
<xml_diff>
--- a/samples/Payslip_Template.xlsx
+++ b/samples/Payslip_Template.xlsx
@@ -587,10 +587,10 @@
         <v>Message Text</v>
       </c>
       <c r="B17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {name}, your payslip for {period} is attached. {password_hint}
-This document contains personal data; please do not forward it.
-عزيزي {name}، مرفق قسيمة راتبك لشهر {period}. {password_hint_ar}
-هذا المستند يحتوي على بيانات شخصية، يرجى عدم مشاركته.</v>
+        <v xml:space="preserve">Dear {name},
+Please find attached your payslip for {period}.
+{password_hint}
+{company}</v>
       </c>
       <c r="C17" t="str">
         <v>Optional. Body of the email / WhatsApp message. Placeholders: {name} {period} {company} {net} {password_hint} {password_hint_ar}</v>
@@ -601,10 +601,10 @@
         <v>Password Rule</v>
       </c>
       <c r="B18" t="str">
-        <v>id+dob</v>
+        <v>id</v>
       </c>
       <c r="C18" t="str">
-        <v>Optional. How each PDF password is built: none, id (National ID / Iqama), id+dob (ID + birth day and month DDMM), dob (DDMMYYYY), custom (uses the "Payslip Password" column). Example: id+dob</v>
+        <v>Optional. PDF password: id (National ID / Iqama number, default), id+dob (ID + birth day and month DDMM), dob (DDMMYYYY), custom (uses the "Payslip Password" column), none. Example: id</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Fix one-line email body; shorter default message
- Settings parser kept collapsing the line breaks of the Message Text
  cell; multiline settings now preserve them
- .eml drafts carry an HTML-only body so Outlook renders paragraphs
- default message: "Dear {first_name}, ... Password: your Iqama number.
  Best regards"; saved copies of older defaults are upgraded
- {first_name} placeholder; shorter password hints

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016bCq81BBBapftKyzt9FyKX
</commit_message>
<xml_diff>
--- a/samples/Payslip_Template.xlsx
+++ b/samples/Payslip_Template.xlsx
@@ -587,13 +587,13 @@
         <v>Message Text</v>
       </c>
       <c r="B17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dear {name},
+        <v xml:space="preserve">Dear {first_name},
 Please find attached your payslip for {period}.
 {password_hint}
-{company}</v>
+Best regards</v>
       </c>
       <c r="C17" t="str">
-        <v>Optional. Body of the email / WhatsApp message. Placeholders: {name} {period} {company} {net} {password_hint} {password_hint_ar}</v>
+        <v>Optional. Body of the email / WhatsApp message. Placeholders: {first_name} {name} {period} {company} {net} {password_hint} {password_hint_ar}</v>
       </c>
     </row>
     <row r="18">

</xml_diff>